<commit_message>
labels: agtzidis_2020 method named_tool/SPM12 -> described_only, ruled 2026-10-22 after the probe
The author's relabel under CALL 1 v1.5 as clarified in protocol v1.6: SPM12 is named once for the
analysis as a whole and bound to no step; SPM12 moves to the inference arm. Made after seeing the
2026-10-21 probe output and recorded as such in the row's Notes, with the superseded state retained.
</commit_message>
<xml_diff>
--- a/ground_truth/motion_correction_labels_v1.xlsx
+++ b/ground_truth/motion_correction_labels_v1.xlsx
@@ -1090,14 +1090,10 @@
       </c>
       <c r="B2" s="7" t="inlineStr">
         <is>
-          <t>named_tool</t>
-        </is>
-      </c>
-      <c r="C2" s="7" t="inlineStr">
-        <is>
-          <t>SPM12</t>
-        </is>
-      </c>
+          <t>described_only</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="n"/>
       <c r="D2" s="8" t="inlineStr">
         <is>
           <t>"performed with SPM12 using Matlab 9.2 … The process comprised realigning the functional data to the mean image of each session"</t>
@@ -1145,7 +1141,11 @@
       <c r="P2" s="8" t="n"/>
       <c r="Q2" s="7" t="inlineStr">
         <is>
-          <t>co-adjudicated. Realignment identified as motion correction (SPM Realign) in consultation; four clauses adjudicated to four separate steps.</t>
+          <t>co-adjudicated. Realignment identified as motion correction (SPM Realign) in consultation; four clauses adjudicated to four separate steps.
+2026-10-22 RELABEL, method named_tool (SPM12) → described_only. Ruled by the author after seeing the motion probe v1 output; co-adjudicated — assistant located the sentence and set out the binding question, author ruled (§7).
+CALL 1 v1.5 binding test, as clarified in protocol v1.6: SPM12 is named once, for the analysis as a whole ("The fMRI data analysis was performed with SPM12 using Matlab 9.2."), and no tool is bound to the realignment, which the paper describes in its own voice. Same shape as derosa's FSL. SPM12 belongs on the inference arm, not the extraction arm; the earlier "SPM Realign" identification was an inference, not a report.
+COBIDAS §4.3 p.10 models step-level attribution ("SPM's realign tool"). That sentence is framed for papers combining tools, so the named_tool reading was defensible.
+Superseded: method_state = named_tool, method_value = SPM12.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
labels: liu_2013 method described_only -> deferred under CALL 11, quote extended, dated note
The author's relabel (workbook row 10): the method defers to the FCP analysis scripts (Biswal 2010);
the quote now carries the deferring sentence with the operation sentence, contiguous verbatim; the
Notes entry records that the rule was adopted before the version-3 run (Amendment 7 pre-declared the
relabel) and the edit made after, co-adjudicated, with the superseded values. Method states now read
deferred 8, named_tool 7, described_only 4.
</commit_message>
<xml_diff>
--- a/ground_truth/motion_correction_labels_v1.xlsx
+++ b/ground_truth/motion_correction_labels_v1.xlsx
@@ -1621,13 +1621,13 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>described_only</t>
+          <t>deferred</t>
         </is>
       </c>
       <c r="C10" s="7" t="n"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>The typical pre-processing steps for the analysis of resting state data were applied, including image coregistration to correct for head motion,</t>
+          <t>FCP analysis scripts (version 1.1-beta, available at http://www.nitrc.org/frs/shownotes.php?release_id=938) (Biswal et al., 2010), which employs AFNI (Cox, 1996) and FSL (http://www.fmrib.ox.ac.uk/fsl/) (Smith et al., 2004) software packages, were used to pre-process the fMRI signals (with minor modifications, described below). The typical pre-processing steps for the analysis of resting state data were applied, including image coregistration to correct for head motion,</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
@@ -1666,7 +1666,15 @@
         </is>
       </c>
       <c r="P10" s="7" t="n"/>
-      <c r="Q10" s="7" t="n"/>
+      <c r="Q10" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-26 RELABEL, method described_only → deferred (target: FCP analysis scripts v1.1-beta, Biswal et al. 2010; target_kind pipeline). Rule adopted by the author on 2026-10-26 BEFORE the motion probe v3 run (prereg Amendment 7 pre-declared this relabel as pending); the edit was made after the run. Co-adjudicated — assistant located the citation sentence and proposed the rule, author ruled (§7).
+CALL 11 (protocol v1.7): the operation is named under a cited pipeline (“FCP analysis scripts … (Biswal et al., 2010) … were used to pre-process the fMRI signals … including image coregistration to correct for head motion”) and the paper states none of the four details (algorithm, transform type, reference image, cost function). Same shape as poldrack’s ref 45. AFNI and FSL are named as the packages the scripts employ, not bound to this step (CALL 1 v1.6). The EPI-to-anatomical registration (align_epi_anat.py, Saad et al. 2009) is a different D.3 row (CALL 2) and does not bear on this bullet.
+method_quote extended to include the deferring sentence (contiguous verbatim text, line breaks joined).
+Sub-items E–P left at not_reported pending the author’s ruling on whether a deferred method carries its unstated sub-items as deferred (poldrack’s pattern: deferred unless stated in-paper).
+Superseded: method_state = described_only; method_quote = the single operation sentence.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="6" t="inlineStr">

</xml_diff>

<commit_message>
labels: liu_2013 second edit -- method_value "FCP analysis scripts" and the six sub-items deferred, dated note
The author's edit (workbook row 10): the pipeline name in method_value, as chen, oconnor, vanderwal
and weber carry it; bullets 2-7 deferred under CALL 7's bullet-level default, none stated in-paper;
the Notes paragraph supersedes the "pending" one with the original text kept. All eight deferred
rows now follow the same pattern; poldrack remains the only one with in-paper overrides. §7's list
is unchanged (same flag, same paper), so no protocol edit.
</commit_message>
<xml_diff>
--- a/ground_truth/motion_correction_labels_v1.xlsx
+++ b/ground_truth/motion_correction_labels_v1.xlsx
@@ -1624,7 +1624,11 @@
           <t>deferred</t>
         </is>
       </c>
-      <c r="C10" s="7" t="n"/>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>FCP analysis scripts</t>
+        </is>
+      </c>
       <c r="D10" t="inlineStr">
         <is>
           <t>FCP analysis scripts (version 1.1-beta, available at http://www.nitrc.org/frs/shownotes.php?release_id=938) (Biswal et al., 2010), which employs AFNI (Cox, 1996) and FSL (http://www.fmrib.ox.ac.uk/fsl/) (Smith et al., 2004) software packages, were used to pre-process the fMRI signals (with minor modifications, described below). The typical pre-processing steps for the analysis of resting state data were applied, including image coregistration to correct for head motion,</t>
@@ -1632,37 +1636,37 @@
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>not_reported</t>
+          <t>deferred</t>
         </is>
       </c>
       <c r="F10" s="7" t="n"/>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>not_reported</t>
+          <t>deferred</t>
         </is>
       </c>
       <c r="H10" s="7" t="n"/>
       <c r="I10" s="7" t="inlineStr">
         <is>
-          <t>not_reported</t>
+          <t>deferred</t>
         </is>
       </c>
       <c r="J10" s="7" t="n"/>
       <c r="K10" s="7" t="inlineStr">
         <is>
-          <t>not_reported</t>
+          <t>deferred</t>
         </is>
       </c>
       <c r="L10" s="7" t="n"/>
       <c r="M10" s="7" t="inlineStr">
         <is>
-          <t>not_reported</t>
+          <t>deferred</t>
         </is>
       </c>
       <c r="N10" s="7" t="n"/>
       <c r="O10" s="7" t="inlineStr">
         <is>
-          <t>not_reported</t>
+          <t>deferred</t>
         </is>
       </c>
       <c r="P10" s="7" t="n"/>
@@ -1672,7 +1676,8 @@
 CALL 11 (protocol v1.7): the operation is named under a cited pipeline (“FCP analysis scripts … (Biswal et al., 2010) … were used to pre-process the fMRI signals … including image coregistration to correct for head motion”) and the paper states none of the four details (algorithm, transform type, reference image, cost function). Same shape as poldrack’s ref 45. AFNI and FSL are named as the packages the scripts employ, not bound to this step (CALL 1 v1.6). The EPI-to-anatomical registration (align_epi_anat.py, Saad et al. 2009) is a different D.3 row (CALL 2) and does not bear on this bullet.
 method_quote extended to include the deferring sentence (contiguous verbatim text, line breaks joined).
 Sub-items E–P left at not_reported pending the author’s ruling on whether a deferred method carries its unstated sub-items as deferred (poldrack’s pattern: deferred unless stated in-paper).
-Superseded: method_state = described_only; method_quote = the single operation sentence.</t>
+Superseded: method_state = described_only; method_quote = the single operation sentence.
+2026-10-26, second edit (same day, after the first): method_value = FCP analysis scripts, the pipeline-name convention the other named-pipeline deferred rows carry (chen CCS; oconnor, vanderwal, weber CPAC). Sub-items E–P not_reported → deferred under CALL 7’s bullet-level default, as applied in all seven other deferred rows; none of the six is stated in-paper (no transform type, fieldmap, reference image, similarity metric, combined-interpolation statement or slice-to-volume statement; the 3 mm MNI resampling is a separate step, not a combined-transform statement). Ruled by the author; edit by the assistant. This supersedes the “pending” paragraph above. Superseded: method_value = (empty); E, G, I, K, M, O = not_reported.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
labels: column R filled on 3 of 3 held-out rows by the author; the v1.8 label pass complete on all 19 rows (sha256 350331c8..., 26,822 bytes; staged blob verified); states unchanged (named_tool 9, deferred 8, described_only 2); cells B, C and R read by id only, D and Q unread
</commit_message>
<xml_diff>
--- a/ground_truth/motion_correction_labels_v1.xlsx
+++ b/ground_truth/motion_correction_labels_v1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cwook/Documents/neurorepro/fmri-repro-agent/ground_truth/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7410FF3A-3A2D-CB4A-AFEC-B63EC7AC7A28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E1F60AA-7794-6D44-9AD6-54B7B455C844}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="19880" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="166">
   <si>
     <t>paper_id</t>
   </si>
@@ -2042,6 +2042,9 @@
       <c r="Q15" s="7" t="s">
         <v>85</v>
       </c>
+      <c r="R15" s="9" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="16" spans="1:18" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="6" t="s">

</xml_diff>